<commit_message>
feat: implement comprehensive attendance management, face detection, and HRMS deployment modules
</commit_message>
<xml_diff>
--- a/deploy/SoftwizApp/backend/data/resumes_data.xlsx
+++ b/deploy/SoftwizApp/backend/data/resumes_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2097,6 +2097,41 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Pruthiraj Swain</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>pruthirajswain1999@gmail.com</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1 6371845225</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Python, Sql, JavaScript, React, Django, Tailwind, Mysql, Sqlite, Visual Studio Code, Git, GitHub, Oop Dsa Os Cn Dbms Restapi Sdlc Agile</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/e14bb5ec-df6e-4eb6-a844-a3c845da4673_pruthiraj_cv_N.pdf</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-06-22T07:01:25.260493</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed candidate resume open issue
</commit_message>
<xml_diff>
--- a/deploy/SoftwizApp/backend/data/resumes_data.xlsx
+++ b/deploy/SoftwizApp/backend/data/resumes_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2132,6 +2132,76 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Rajwinder Rani</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>krajwinderk909@gmail.com</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>+919780922617</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Portals., Synthesis, Feb, Oct, Business, Executive, Portals, Handling, Social, Media, Platforms, Multi, Tasking, Sep, Jan, Critical, Thinking, Lead, Generation, Designing, Solutions, Autocad, Bidding, In, Different, Telecom, Fibers, Plan, Auto, Cad, Hfci, Design, Google, Search, For, Data, Creative, Mining, Tree, English, Hindi</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/e367d6a6-b4fe-4be9-826b-df231e1231c0_Rajwinder_Resume_.pdf</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-06-23T09:08:59.419323</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Anish Yadav</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>anishyaduvanshee@gmail.com</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>+919506070868</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Academic, Computer, Foundation, Technical, Readiness, It, Typing, Speed, Office, Automation, Microsoft Office, Ms, Word, Excel, Power, Point, Data, Entry, E Availability</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/33b88b2b-da9e-4b67-86dd-9cab8f196f7f_anish_doc_resume.docx</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-06-23T09:34:08.234610</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add check-in checkout function
</commit_message>
<xml_diff>
--- a/deploy/SoftwizApp/backend/data/resumes_data.xlsx
+++ b/deploy/SoftwizApp/backend/data/resumes_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2202,6 +2202,68 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>phanindra.chikkala@gmail.com</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>+919133472694</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>["JavaScript", "Postman", "Java", "Database: Mysql", "GitHub", "VS Code", "Eclipse Ide", "Npm", "Oop", "Mvc Architecture", "Crud Operations"]</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/96891beb-7ed7-451f-8dae-3823566c0c9a_Phanindra_Resume-1.pdf</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-06-24T04:56:10.604298</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>shamsingsainin@gmail.com</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>+919815448010</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>["Shamsingsainin@Gmail.Com", "And Follow-Ups.", "And Certifications.", "And Presentations.", "And Virtual Events.", "Punjab", "Marketing", "Digital Marketing", "Strong", "Sales", "Ed-Tech Division", "Qualification", "Training Programs", "Emailers", "Brochures", "Demo Sessions", "Patiala", "Qualifying Leads", "Public Speaking", "And Pitching", "Excel", "Nationality: Indian", "English", "Hindi", "Punjabi", "Hobbies: Travelling", "Swimming", "Physical Fitness", "Additional Information"]</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/8853802f-5a21-49a2-8c09-9071bdeb0e7e_36f00a59-ba2a-4551-a054-c5c6becfe149_Sham_Singh_Resume_26.pdf</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-06-24T11:04:04.663252</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add cctv camera functionality
</commit_message>
<xml_diff>
--- a/deploy/SoftwizApp/backend/data/resumes_data.xlsx
+++ b/deploy/SoftwizApp/backend/data/resumes_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2264,6 +2264,568 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>neelamjharbade94@gmail.com</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>+919302545725</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>["Best Of My Knowledge.", "And Concepts", "Other Knowledge", "Hobbies", " Travelling", "Strength", " Confident", " Punctual", "2-Personal Information", "English", "Declaration", "Date :"]</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/1180aade-aad9-4413-b475-66f601969afb_neelam_new_word_file_2026__1_.pdf</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:02:19.913456</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Navjot Singh</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>+919056244877</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>["Innovate Pvt. Ltd.", "And Cheesy Crazy Cafe.", "Blender", "And Visual Innovation.", "Punjab", "Mohali", "India", "And Lbm", "Promotional Campaigns", "Promotional Reels", "Editing", "Sound Selection", "Transitions", "And Post", "Lets Rentz", "Video Advertisements", "Cgi Visuals", "Digital Advertisements", "Visual Assets", "After Effects", "Higgsfield"]</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/7e69a409-40d2-4b00-8717-6f79eb080365_Navjot_Singh_-_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:11:18.994390</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>["Camscanner"]</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/548ca651-b14e-4a4e-bd1b-885a2681314f_ResumeLakshayDhawan.pdf</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:15:00.840703</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Navjot Singh</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>+919056244877</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>["Innovate Pvt. Ltd.", "And Cheesy Crazy Cafe.", "Blender", "And Visual Innovation.", "Punjab", "Mohali", "India", "And Lbm", "Promotional Campaigns", "Promotional Reels", "Editing", "Sound Selection", "Transitions", "And Post", "Lets Rentz", "Video Advertisements", "Cgi Visuals", "Digital Advertisements", "Visual Assets", "After Effects", "Higgsfield"]</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/e80d56de-92e0-4d7d-b5e2-7c6efbbd745d_Navjot_Singh_-_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:25:28.591103</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Navjot Singh</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>+919056244877</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>["Innovate Pvt. Ltd.", "And Cheesy Crazy Cafe.", "Blender", "And Visual Innovation.", "Punjab", "Mohali", "India", "And Lbm", "Promotional Campaigns", "Promotional Reels", "Editing", "Sound Selection", "Transitions", "And Post", "Lets Rentz", "Video Advertisements", "Cgi Visuals", "Digital Advertisements", "Visual Assets", "After Effects", "Higgsfield"]</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/b3dac8b5-36ba-427b-94d9-87a573ab9ef4_Navjot_Singh_-_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:42:38.467813</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Navjot Singh</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>+919056244877</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>["Innovate Pvt. Ltd.", "And Cheesy Crazy Cafe.", "Blender", "And Visual Innovation.", "Punjab", "Mohali", "India", "And Lbm", "Promotional Campaigns", "Promotional Reels", "Editing", "Sound Selection", "Transitions", "And Post", "Lets Rentz", "Video Advertisements", "Cgi Visuals", "Digital Advertisements", "Visual Assets", "After Effects", "Higgsfield"]</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/dbe62ae8-a118-4243-abe7-d4a70ce82a58_Navjot_Singh_-_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:53:12.563475</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>["Camscanner"]</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/0c16e016-3071-4524-8864-96c93ba2b0d1_ResumeLakshayDhawan.pdf</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:53:22.716009</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Navjot Singh</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>+919056244877</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>["Innovate Pvt. Ltd.", "And Cheesy Crazy Cafe.", "Blender", "And Visual Innovation.", "Punjab", "Mohali", "India", "And Lbm", "Promotional Campaigns", "Promotional Reels", "Editing", "Sound Selection", "Transitions", "And Post", "Lets Rentz", "Video Advertisements", "Cgi Visuals", "Digital Advertisements", "Visual Assets", "After Effects", "Higgsfield"]</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/22a83756-8b96-415b-a35f-03532e6911d9_Navjot_Singh_-_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-06-24T12:58:00.295293</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Ritesh Sharma</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>riteshs944@gmail.com</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>+919882082640</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>["Hindi", "English", "Reading", "Playing", "Cooking", "Gaming", "Coding"]</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/563837e1-d671-4dff-a2f5-dba5715e5053_87cef32d-9c03-44d7-81bb-af7611374fda_ResumeRiteshKumar.pdf</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-06-25T04:55:21.237494</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Kavya</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>kavyagauri2003@gmail.com</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>+916393428787</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>["Forums/Marketplaces", "React", "JavaScript", "Mongodb", "Python", "Technology", "Fast", "Access", "Login", "Users", "Courses", "(Pause", "Play", "Nodes", "(Numpy", "Pandas", "Scikit-Learn)", "Forest", "Structures", "Algorithms", "Systems", "(Oops)", "Hackathon", "Head", "Branch", "Fest", "Branding", "Design", "Member", "Club", "Ideation"]</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/4f5831fd-5bcd-49e7-be3b-b7bf24b2ecf1_KAVYA_GAURI.pdf</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-06-25T04:56:55.357999</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Prasoon Kumar</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>prasoonkumar030@gmail.com</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>+916299730974</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>["Intellij Idea", "VS Code", "Computer Networks", "Pandas", "Scikit-Learn", "Mongodb", "Flask", "JavaScript", "Node.Js", "Python", "Express.Js", "GitHub", "Sql", "Oracle", "Express", "React", "Java", "Git", "Intellij", "Mysql"]</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/f6290092-2216-48d3-af07-eb5d1b529e21_Prasoon_Kumar_Resume_final-1.pdf</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-06-25T06:40:09.367330</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Result Awaited</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>rajputpooja0920@gmail.com</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>+917814084208</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>["Hard Working"]</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/620d1071-4131-4ec3-9715-6e0a2502278c_RESUME_POOJA.pdf</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-06-25T06:40:09.905558</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/0ff91059-5958-4ee2-8254-6435dd58bc88_ResumeLakshayDhawan.pdf</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-06-25T07:38:42.072684</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>amansharma8401@gmail.com</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>+917009989542</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>["Laravel"]</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/fe52cf32-e1ba-4cec-b788-ae832d9cbf47_Aman-SharmaCV.pdf</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-06-25T07:55:37.182721</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Prabal Kaslotra</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>guptaprabalkaslotra@gmail.com</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>+916005659048</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>["Code.", "Process.", "View", "For Password Updates Every 6 Months.", "Streamlining The Order And Checkout", "Which Automated The Process Of", "And Built Custom Solutions", "And Easy To Maintain.", "And Track Team Hierarchy.", "Clean User Interfaces", "Specific Client Needs.", "Including Admin Dashboards", "Dynamic Form Handling.", "Managing Customer Billing", "And Database Connectivity.", "Calculating Total Bills", "Tailored To", "Allowing Clients", "More Reliable", "Admin Panels.", "Where Applicable.", "Progress Updates.", "Room Reservations", "And Payments.", "And Generating", "Version Control:", "Efficient", "Operations.", "Status", "Reusable", "Internship", "Planning.", "Reports.", "Databases:", "Tools Like Git And Always Aim To Write Code That’S Clean", "And Managing Databases. I’M Comfortable With Version Control", " Integrated Multiple Shipping And Payment Gateways", "To Store And Manage Product/Media Files Efficiently.", "Frontend And Node.Js With Express.Js For Backend.", "The Brihaspati Infotech Pvt Ltd", "Pg Tech. Pvt. Ltd Sec-34A", " Built Several Real-World Projects", "March 2024 – Present", "September 2023 – February", "Full Stack Development Intern", "Esteplogic It Solutions", "User-Friendly Storefronts And", "And Interactive Uis.", "Java Developer Intern", "Java Gui Development", " Restful Apis", "Punjab Computer Science", "Jammu Computer Science", "Connecting Apis", "Like Faire.", "Data-Driven Applications", "Mongodb Integration", "Nielt Jammu", "Frontend Development:", "Backend Development:", "E-Commerce Platforms:", "Api Integrations", "Languages Known", " Shopify", " Git", " Mysql", " English", " Hindi", " Dogri", " Punjabi", "Chandigarh", "JavaScript", "Jquery", "Bootstrap", "Laravel", "Yii", "Cs-Cart", "Wordpress", "Others:", "Https://In.Linkedin.Com/In/Prabalkaslotra", "(Swing/Javafx)", "Engineering"]</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/febaf283-090a-49e0-85c0-77c302ed132b_Prabal_Kaslotra_Updated_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-06-25T10:40:15.329483</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>itstusharkumar15@gmail.com</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>+918194846705</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>["Performance", "Infrastructure", "And Rapid Issue Resolution Based On Client Requirements.", "And New Features Under Tight Deadlines.", "Server", "Domains", "Testing", "Security", "Order", "Debugging", "Data From Databases Without Writing Complex Queries.", "Optimized Database Layer For Evolving Needs.", "And Deployment Best Practices.", "And Maintained Frontend Applications.", "And Production Environment Management.", "Managing Production Deployments", "And Migration Scripts", "Delivered Bug Fixes", "And Customer Engagement", "And Product Images.", "And Featured Products.", "Dataset Curation", "Performance Improvements", "Enhancing Functionality", "Server Infrastructure", "Including Categories", "And Migrations", "Performance Optimizations", "Product Management", "Developing", "Deploying", "Reliability", "Processing", "Pricing", "Inventory", "Offers", "Optimization", "Designed", "Quick And Simple Store Setup With Minimal Configuration.", "And Cloudflare Services. Skilled In Frontend Development", "Published Technical Blogs On Ai Model Selection", "Providing An Easy-To-Use Interface For Store Setup", "Real-Time Analytics And Reporting For Business Insights.", "Distilbert) With Curated Datasets To Improve Accuracy.", "Published Technical Blogs And Delivered Bug Fixes", "Researched And Integrated Ai/Nlp Models (Gpt-", "Full Stack Developer 11/2024 – 01/", "Contributed To B2B Spice Web Platform", "Collaborated With Team To Deliver Efficient", "Full Stack Developer 06/2025 – 06/", "Pksoft E-Commerce Platform 06/2025 – 06/", "Secure Order Management And Tracking System.", "Seo-Friendly Architecture To Improve Online Visibility.", "Hr Ai Chatbot 02/2025 – 05/", "Zeusinfinity Services 02/2025 – 05/", "Promotional Features Such As Discounts", "Queries And Automated Db-To-Excel Sync.", "Easy Product Catalog Management", "And Python Rest Api", "Integrated Gpt-2/Distilbert For Nlp", "Integrated Nlp Models (Gpt-", "Designed Postgresql Schemas", "Maintainable Full-Stack Solutions.", "And Cloudflare Configurations.", "Tech Intern", "Fooz Food", "Restful Apis", "Full-Stack Developer", "Frontend Engineer", "Built Responsive", "Performed Testing", "AI", "React", "Node.Js", "Abohar", "Mongodb", "Python", "Cloudflare"]</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/c872fa5b-3b05-40d6-bcfe-245a8a52c6aa_Tushar_Kumar_FlowCV_Resume_2026-06-21.pdf</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-06-25T10:49:01.221551</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Akshit Sood</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>akshitsood978@gmail.com</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>+918005829304</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>["Microservices", "Azure Functions", "VS Code", "Azure Devops", "Asp.Net Core", "Github Actions", "Asp.Net Mvc", "Rest Api", "Entity Framework", "SQL Server", "Visual Studio", "Azure", "Lambda", "Dynamodb", "Jira", "Postgresql", "Bitbucket", "Git", "Postman", "S3", "Swagger", "Openapi", "Scrum", "Agile", "Redis", "Json", "Ec2", "Mysql", "JavaScript", "Devops", "GitHub"]</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/7c4ed1c1-a64e-4d33-b515-abec474fd6a4_Akshit_Sood_CV.pdf</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-06-25T11:46:26.023727</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Sakshi Dangi</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>sakshidangi002@gmail.com</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>+917807592508</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>["Web", "Langchain", "Fastapi", "Flask", "Scrum", "Postgresql", "Python", "JavaScript", "Uml", "Built", "Present", "TypeScript", "Java"]</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>http://127.0.0.1:8501/files/2e7c4969-ca93-4620-9753-357205ef49c8_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-06-25T12:16:03.550795</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>